<commit_message>
data analysis for ePCD
</commit_message>
<xml_diff>
--- a/courses/nano/semi/docs/gregorio-jaca-peter-tallosy_ePCD/ePCD_meas_info.xlsx
+++ b/courses/nano/semi/docs/gregorio-jaca-peter-tallosy_ePCD/ePCD_meas_info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\HallgatoiLabor\Labor\wagner_szomtagh_csoma_ePCD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grego\OneDrive\Documents\BME_UNI_WORK\petya\physeng_lab_reports\courses\nano\semi\docs\gregorio-jaca-peter-tallosy_ePCD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A001F4AC-B968-452D-9518-8B36E7E04919}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0308FB19-CF1E-42F9-AC36-350523DF1017}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5115" yWindow="1695" windowWidth="20790" windowHeight="13005" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="19704" windowHeight="10479" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -320,8 +320,9 @@
       <family val="1"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -710,8 +711,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -764,7 +766,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -777,8 +778,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1058,9 +1061,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.28515625" bestFit="1" customWidth="1"/>
@@ -1069,12 +1072,12 @@
     <col min="11" max="11" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="16.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="16.600000000000001" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>69</v>
       </c>
@@ -1090,13 +1093,13 @@
       <c r="G2" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="I2" s="29" t="s">
+      <c r="I2" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
-    </row>
-    <row r="3" spans="1:11" ht="14.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
+    </row>
+    <row r="3" spans="1:11" ht="14.3" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="25" t="s">
         <v>64</v>
       </c>
@@ -1112,13 +1115,13 @@
       <c r="G3" s="13">
         <v>21</v>
       </c>
-      <c r="I3" s="30" t="s">
+      <c r="I3" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="J3" s="31"/>
-      <c r="K3" s="32"/>
-    </row>
-    <row r="4" spans="1:11" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J3" s="30"/>
+      <c r="K3" s="31"/>
+    </row>
+    <row r="4" spans="1:11" ht="17.850000000000001" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="26" t="s">
         <v>65</v>
       </c>
@@ -1144,7 +1147,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="26" t="s">
         <v>66</v>
       </c>
@@ -1170,7 +1173,7 @@
         <v>3690000000000000</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
         <v>67</v>
       </c>
@@ -1196,7 +1199,7 @@
         <v>2020000000000000</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="15.7" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="27" t="s">
         <v>68</v>
       </c>
@@ -1222,7 +1225,7 @@
         <v>1540000000000000</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>73</v>
       </c>
@@ -1245,7 +1248,7 @@
         <v>1460000000000000</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>74</v>
       </c>
@@ -1265,7 +1268,7 @@
         <v>1390000000000000</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="15.7" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F10" s="16" t="s">
         <v>62</v>
       </c>
@@ -1282,7 +1285,7 @@
         <v>1460000000000000</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="15.7" thickTop="1" x14ac:dyDescent="0.25">
       <c r="I11" s="2" t="s">
         <v>16</v>
       </c>
@@ -1293,7 +1296,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -1310,7 +1313,7 @@
         <v>1560000000000000</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -1333,7 +1336,7 @@
         <v>1740000000000000</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1356,7 +1359,7 @@
         <v>1840000000000000</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="I15" s="2" t="s">
         <v>21</v>
       </c>
@@ -1371,7 +1374,7 @@
       <c r="A16" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="28" t="s">
+      <c r="B16" s="32" t="s">
         <v>4</v>
       </c>
       <c r="I16" s="2" t="s">
@@ -1384,7 +1387,7 @@
         <v>2070000000000000</v>
       </c>
     </row>
-    <row r="17" spans="9:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="9:11" ht="15" x14ac:dyDescent="0.25">
       <c r="I17" s="2" t="s">
         <v>23</v>
       </c>
@@ -1395,7 +1398,7 @@
         <v>2140000000000000</v>
       </c>
     </row>
-    <row r="18" spans="9:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="9:11" ht="15" x14ac:dyDescent="0.25">
       <c r="I18" s="2" t="s">
         <v>24</v>
       </c>
@@ -1692,7 +1695,7 @@
         <v>1940000000000000</v>
       </c>
     </row>
-    <row r="45" spans="9:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="9:11" ht="15" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I45" s="6" t="s">
         <v>51</v>
       </c>
@@ -1708,7 +1711,10 @@
     <mergeCell ref="I2:K2"/>
     <mergeCell ref="I3:K3"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B16" r:id="rId1" xr:uid="{2A68D7AF-A74F-4BF5-8E35-F1845A920D2D}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>